<commit_message>
tested with mock now integerated real with IP and my_plc.py
</commit_message>
<xml_diff>
--- a/TipDressBackup/18-10-2025.xlsx
+++ b/TipDressBackup/18-10-2025.xlsx
@@ -443,10 +443,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C2" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -456,10 +456,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="C3" t="n">
-        <v>67</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -469,10 +469,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="C4" t="n">
-        <v>94</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>